<commit_message>
updated some sims and plots
</commit_message>
<xml_diff>
--- a/EXP_5/READINGS/DIFF_AMPLIFIER/EXP.xlsx
+++ b/EXP_5/READINGS/DIFF_AMPLIFIER/EXP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EDC_LAB\EXP_5\READINGS\DIFF_AMPLIFIER\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2361CD-6A4B-4646-AF4E-2F032DA4E3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15725127-8F10-4705-B973-F44F1965A1F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A82E2911-34DA-46EE-B228-885B7FB33E27}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A82E2911-34DA-46EE-B228-885B7FB33E27}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -481,6 +481,1324 @@
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>VD1 &amp; VD2 vs Vid</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>VD1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-0.30000000000000027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.27</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.24000000000000021</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.18000000000000016</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3.0000000000000249E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.9999999999999805E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.17999999999999972</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.23999999999999977</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.27</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.29999999999999982</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$C$2:$C$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>6.35</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.09</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.83</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.59</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.36</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.1100000000000003</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.87</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.6100000000000003</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.32</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.84</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.57</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.33</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2.27</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2.25</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2.2400000000000002</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>2.2400000000000002</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>2.23</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>2.23</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>2.23</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>2.23</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-AE40-488D-9151-B43E160B3EFA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>VD2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-0.30000000000000027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.27</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.24000000000000021</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.18000000000000016</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3.0000000000000249E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.9999999999999805E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.17999999999999972</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.23999999999999977</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.27</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.29999999999999982</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$D$2:$D$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>1.95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.97</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.99</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.02</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.0499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.06</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.16</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.2599999999999998</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.5499999999999998</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3.43</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.71</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3.75</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3.76</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.77</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.77</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.77</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>3.77</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>3.78</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>3.78</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-AE40-488D-9151-B43E160B3EFA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1987823216"/>
+        <c:axId val="1814541680"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1987823216"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1814541680"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1814541680"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1987823216"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>ID1 &amp; ID2 vs Vid</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ID1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-0.30000000000000027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.27</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.24000000000000021</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.18000000000000016</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3.0000000000000249E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.9999999999999805E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.17999999999999972</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.23999999999999977</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.27</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.29999999999999982</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$E$2:$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>3.138888888888889E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.2833333333333332E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.4277777777777775E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5611111111111114E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.6888888888888888E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.8277777777777779E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.9611111111111111E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>4.1055555555555553E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>4.2666666666666665E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4.5333333333333337E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>5.2388888888888888E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>5.372222222222222E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.4055555555555558E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5.4166666666666669E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>5.422222222222222E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>5.422222222222222E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>5.4277777777777772E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5.4277777777777772E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>5.4277777777777772E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>5.4277777777777772E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-84DA-43CC-8C65-7F734FAC229B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet3!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ID2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$B$2:$B$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>-0.30000000000000027</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.27</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.24000000000000021</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.18000000000000016</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>-8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-3.0000000000000249E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.9999999999999805E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.0000000000000053E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>8.9999999999999858E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.12000000000000011</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.14999999999999991</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.17999999999999972</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.20999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.23999999999999977</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.27</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.29999999999999982</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$F$2:$F$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="20"/>
+                <c:pt idx="0">
+                  <c:v>5.5833333333333339E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.5722222222222222E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.5611111111111111E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.5444444444444449E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.5277777777777773E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.5222222222222221E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5.5E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.4666666666666669E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>5.411111111111111E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.2499999999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>4.7611111111111111E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4.6055555555555551E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>4.583333333333333E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>4.5777777777777778E-2</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>4.5722222222222227E-2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4.5722222222222227E-2</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4.5722222222222227E-2</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.5722222222222227E-2</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4.5666666666666668E-2</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.5666666666666668E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-84DA-43CC-8C65-7F734FAC229B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1981438928"/>
+        <c:axId val="1982159152"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1981438928"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1982159152"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1982159152"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1981438928"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2627,6 +3945,336 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>VRSS(RSS=22)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet2!$A$2:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet2!$D$2:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.17</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.63</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4199-4797-8CE8-CB3A75DF51CB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1987800944"/>
+        <c:axId val="1814535920"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1987800944"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1814535920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1814535920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1987800944"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
@@ -2992,7 +4640,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3406,6 +5054,86 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3725,6 +5453,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -4241,7 +6009,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4757,7 +6525,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -5273,7 +7041,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -5789,7 +7557,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6305,7 +8073,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6821,7 +8589,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -7337,7 +9105,1555 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -8076,6 +11392,42 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>156210</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>156210</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA25E94B-756D-E4B9-68D4-8237B0E2F9F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8148,6 +11500,78 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E75E0C2-7B2F-5A33-5AD0-05BD54D989DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>289560</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>594360</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3549DF3-D11A-D95B-35CC-AB8D90E47AFC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>